<commit_message>
Add Scenarios driver notes in column B with colon formatting
Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/model18_wsp_formulas.xlsx
+++ b/LULU/model18_wsp_formulas.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Cover" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="WACC" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Scenarios" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Revenue Drivers" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="DCF" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Comps" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WACC" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revenue Drivers" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comps" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -30,7 +30,7 @@
     <numFmt numFmtId="169" formatCode="0.0x"/>
     <numFmt numFmtId="170" formatCode="0.0"/>
   </numFmts>
-  <fonts count="58">
+  <fonts count="60">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -369,6 +369,15 @@
       <i val="1"/>
       <sz val="8"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00404040"/>
+      <sz val="9"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -428,7 +437,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="134">
+  <cellXfs count="136">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -789,6 +798,12 @@
     </xf>
     <xf numFmtId="0" fontId="56" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="57" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="58" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="59" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1812,7 +1827,11 @@
           <t>Key assumptions (5-yr forecast)</t>
         </is>
       </c>
-      <c r="B3" s="15" t="n"/>
+      <c r="B3" s="134" t="inlineStr">
+        <is>
+          <t>How it moves</t>
+        </is>
+      </c>
       <c r="C3" s="15" t="inlineStr">
         <is>
           <t>Source (click)</t>
@@ -1826,7 +1845,11 @@
           <t>FY2026E revenue growth</t>
         </is>
       </c>
-      <c r="B4" s="17" t="n"/>
+      <c r="B4" s="135" t="inlineStr">
+        <is>
+          <t>Year-one sales change: bear falls most.</t>
+        </is>
+      </c>
       <c r="C4" s="18" t="inlineStr">
         <is>
           <t>LULU Q2 FY2026 earnings release</t>
@@ -1849,7 +1872,11 @@
           <t>FY2027–FY2030E revenue growth (avg)</t>
         </is>
       </c>
-      <c r="B5" s="17" t="n"/>
+      <c r="B5" s="135" t="inlineStr">
+        <is>
+          <t>Years two-five average growth: bull fastest.</t>
+        </is>
+      </c>
       <c r="C5" s="18" t="inlineStr">
         <is>
           <t>StockAnalysis: LULU 3Y revenue forecast</t>
@@ -1872,7 +1899,11 @@
           <t>Run-rate EBIT margin (clean, ex-refunds)</t>
         </is>
       </c>
-      <c r="B6" s="17" t="n"/>
+      <c r="B6" s="135" t="inlineStr">
+        <is>
+          <t>Starting operating margin before linear ramp.</t>
+        </is>
+      </c>
       <c r="C6" s="18" t="inlineStr">
         <is>
           <t>Q2 FY2026 release: 18.8% OM minus 560bps tariffs</t>
@@ -1895,7 +1926,11 @@
           <t>FY26 IEEPA tariff refunds ($k, already in guide)</t>
         </is>
       </c>
-      <c r="B7" s="17" t="n"/>
+      <c r="B7" s="135" t="inlineStr">
+        <is>
+          <t>One-time year-one EBIT boost: zero after.</t>
+        </is>
+      </c>
       <c r="C7" s="18" t="inlineStr">
         <is>
           <t>Q2 FY2026 release: $134.5M IEEPA tariff refunds</t>
@@ -1918,7 +1953,11 @@
           <t>Terminal (FY2030E) EBIT margin</t>
         </is>
       </c>
-      <c r="B8" s="17" t="n"/>
+      <c r="B8" s="135" t="inlineStr">
+        <is>
+          <t>Year-five target margin after linear ramp.</t>
+        </is>
+      </c>
       <c r="C8" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: Operating margin 19.9% (one hit)</t>
@@ -1941,7 +1980,11 @@
           <t>WACC</t>
         </is>
       </c>
-      <c r="B9" s="17" t="n"/>
+      <c r="B9" s="135" t="inlineStr">
+        <is>
+          <t>Flat discount rate: higher bear, lower bull.</t>
+        </is>
+      </c>
       <c r="C9" s="18" t="inlineStr">
         <is>
           <t>WACC tab: CAPM build</t>
@@ -1965,7 +2008,11 @@
           <t>Terminal growth</t>
         </is>
       </c>
-      <c r="B10" s="17" t="n"/>
+      <c r="B10" s="135" t="inlineStr">
+        <is>
+          <t>Perpetuity growth rate: flat across all years.</t>
+        </is>
+      </c>
       <c r="C10" s="18" t="inlineStr">
         <is>
           <t>FRED: Real GDP (GDPC1)</t>
@@ -1988,7 +2035,11 @@
           <t>Cash tax rate</t>
         </is>
       </c>
-      <c r="B11" s="17" t="n"/>
+      <c r="B11" s="135" t="inlineStr">
+        <is>
+          <t>Flat tax percentage applied every forecast year.</t>
+        </is>
+      </c>
       <c r="C11" s="18" t="inlineStr">
         <is>
           <t>Q2 FY2026 outlook: tax rate ≈ 30%</t>
@@ -2011,7 +2062,11 @@
           <t>D&amp;A % of revenue</t>
         </is>
       </c>
-      <c r="B12" s="17" t="n"/>
+      <c r="B12" s="135" t="inlineStr">
+        <is>
+          <t>Depreciation scales as fixed percent of revenue.</t>
+        </is>
+      </c>
       <c r="C12" s="18" t="inlineStr">
         <is>
           <t>LULU CF statement (10-K)</t>
@@ -2034,7 +2089,11 @@
           <t>Capex % of revenue</t>
         </is>
       </c>
-      <c r="B13" s="19" t="n"/>
+      <c r="B13" s="135" t="inlineStr">
+        <is>
+          <t>Investment scales as fixed percent of revenue.</t>
+        </is>
+      </c>
       <c r="C13" s="38" t="inlineStr">
         <is>
           <t>LULU 10-K: 2026 capex guide $725–745M</t>
@@ -2057,7 +2116,11 @@
           <t>Gross margin %</t>
         </is>
       </c>
-      <c r="B14" s="17" t="n"/>
+      <c r="B14" s="135" t="inlineStr">
+        <is>
+          <t>Merchandise margin held flat every forecast year.</t>
+        </is>
+      </c>
       <c r="C14" s="18" t="inlineStr">
         <is>
           <t>LULU FY2025 10-K: Gross profit &amp; COGS</t>
@@ -2077,10 +2140,14 @@
     <row r="15" ht="150" customHeight="1">
       <c r="A15" s="16" t="inlineStr">
         <is>
-          <t>DSO (days) — flat vs FY25</t>
-        </is>
-      </c>
-      <c r="B15" s="17" t="n"/>
+          <t>DSO (days): flat vs FY25</t>
+        </is>
+      </c>
+      <c r="B15" s="135" t="inlineStr">
+        <is>
+          <t>Collection days held flat near six yearly.</t>
+        </is>
+      </c>
       <c r="C15" s="18" t="inlineStr">
         <is>
           <t>LULU FY2025 10-K: Accounts receivable, net</t>
@@ -2106,7 +2173,11 @@
           <t>FY25 DIO anchor (days)</t>
         </is>
       </c>
-      <c r="B16" s="17" t="n"/>
+      <c r="B16" s="135" t="inlineStr">
+        <is>
+          <t>Starting inventory days before annual decline begins.</t>
+        </is>
+      </c>
       <c r="C16" s="18" t="inlineStr">
         <is>
           <t>LULU FY2025 10-K: Inventories &amp; COGS</t>
@@ -2132,7 +2203,11 @@
           <t>DIO decline (days / forecast yr)</t>
         </is>
       </c>
-      <c r="B17" s="17" t="n"/>
+      <c r="B17" s="135" t="inlineStr">
+        <is>
+          <t>Inventory days fall one day each year.</t>
+        </is>
+      </c>
       <c r="C17" s="18" t="inlineStr">
         <is>
           <t>LULU FY2025 10-K: inventory &amp; markdown outlook</t>
@@ -2152,10 +2227,14 @@
     <row r="18" ht="84" customHeight="1">
       <c r="A18" s="16" t="inlineStr">
         <is>
-          <t>DPO (days) — flat vs FY25</t>
-        </is>
-      </c>
-      <c r="B18" s="17" t="n"/>
+          <t>DPO (days): flat vs FY25</t>
+        </is>
+      </c>
+      <c r="B18" s="135" t="inlineStr">
+        <is>
+          <t>Payment days held flat near twenty-five yearly.</t>
+        </is>
+      </c>
       <c r="C18" s="18" t="inlineStr">
         <is>
           <t>LULU FY2025 10-K: Accounts payable &amp; COGS</t>
@@ -2181,7 +2260,11 @@
           <t>Prepaid expenses (% of revenue)</t>
         </is>
       </c>
-      <c r="B19" s="17" t="n"/>
+      <c r="B19" s="135" t="inlineStr">
+        <is>
+          <t>Other current assets flat percent of revenue.</t>
+        </is>
+      </c>
       <c r="C19" s="18" t="inlineStr">
         <is>
           <t>LULU FY2025 10-K: other current assets (residual)</t>
@@ -2207,7 +2290,11 @@
           <t>Accrued liabilities (% of revenue)</t>
         </is>
       </c>
-      <c r="B20" s="17" t="n"/>
+      <c r="B20" s="135" t="inlineStr">
+        <is>
+          <t>Accrued payables flat percent of revenue.</t>
+        </is>
+      </c>
       <c r="C20" s="18" t="inlineStr">
         <is>
           <t>LULU FY2025 10-K: Accrued liabilities and other</t>
@@ -2233,6 +2320,11 @@
           <t>Pitch CFF: fixed buyback ($k/yr) bear/base</t>
         </is>
       </c>
+      <c r="B21" s="135" t="inlineStr">
+        <is>
+          <t>Bear base retire fixed dollars yearly.</t>
+        </is>
+      </c>
       <c r="F21" s="37" t="n">
         <v>750000</v>
       </c>
@@ -2249,6 +2341,11 @@
           <t>Pitch CFF: % of FCF to buybacks (bull)</t>
         </is>
       </c>
+      <c r="B22" s="135" t="inlineStr">
+        <is>
+          <t>Bull spends set percent of free cash.</t>
+        </is>
+      </c>
       <c r="F22" s="20" t="n">
         <v>0</v>
       </c>
@@ -2259,6 +2356,7 @@
         <v>0.75</v>
       </c>
     </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24" s="14" t="inlineStr">
         <is>
@@ -2269,7 +2367,12 @@
     <row r="25">
       <c r="A25" s="41" t="inlineStr">
         <is>
-          <t>Revenue – year 1</t>
+          <t>Revenue: year 1</t>
+        </is>
+      </c>
+      <c r="B25" s="135" t="inlineStr">
+        <is>
+          <t>Grows or shrinks using scenario-specific growth rates.</t>
         </is>
       </c>
       <c r="F25" s="42">
@@ -2288,7 +2391,7 @@
     <row r="26">
       <c r="A26" s="41" t="inlineStr">
         <is>
-          <t>Revenue – year 2</t>
+          <t>Revenue: year 2</t>
         </is>
       </c>
       <c r="F26" s="42">
@@ -2307,7 +2410,7 @@
     <row r="27">
       <c r="A27" s="41" t="inlineStr">
         <is>
-          <t>Revenue – year 3</t>
+          <t>Revenue: year 3</t>
         </is>
       </c>
       <c r="F27" s="42">
@@ -2326,7 +2429,7 @@
     <row r="28">
       <c r="A28" s="41" t="inlineStr">
         <is>
-          <t>Revenue – year 4</t>
+          <t>Revenue: year 4</t>
         </is>
       </c>
       <c r="F28" s="42">
@@ -2345,7 +2448,7 @@
     <row r="29">
       <c r="A29" s="41" t="inlineStr">
         <is>
-          <t>Revenue – year 5</t>
+          <t>Revenue: year 5</t>
         </is>
       </c>
       <c r="F29" s="42">
@@ -2364,7 +2467,12 @@
     <row r="30">
       <c r="A30" s="41" t="inlineStr">
         <is>
-          <t>Gross margin % – year 1</t>
+          <t>Gross margin %: year 1</t>
+        </is>
+      </c>
+      <c r="B30" s="135" t="inlineStr">
+        <is>
+          <t>Stays flat at scenario margin every year.</t>
         </is>
       </c>
       <c r="F30" s="43">
@@ -2383,7 +2491,7 @@
     <row r="31">
       <c r="A31" s="41" t="inlineStr">
         <is>
-          <t>Gross margin % – year 2</t>
+          <t>Gross margin %: year 2</t>
         </is>
       </c>
       <c r="F31" s="43">
@@ -2402,7 +2510,7 @@
     <row r="32">
       <c r="A32" s="41" t="inlineStr">
         <is>
-          <t>Gross margin % – year 3</t>
+          <t>Gross margin %: year 3</t>
         </is>
       </c>
       <c r="F32" s="43">
@@ -2421,7 +2529,7 @@
     <row r="33">
       <c r="A33" s="41" t="inlineStr">
         <is>
-          <t>Gross margin % – year 4</t>
+          <t>Gross margin %: year 4</t>
         </is>
       </c>
       <c r="F33" s="43">
@@ -2440,7 +2548,7 @@
     <row r="34">
       <c r="A34" s="41" t="inlineStr">
         <is>
-          <t>Gross margin % – year 5</t>
+          <t>Gross margin %: year 5</t>
         </is>
       </c>
       <c r="F34" s="43">
@@ -2459,7 +2567,12 @@
     <row r="35">
       <c r="A35" s="41" t="inlineStr">
         <is>
-          <t>Cost of goods sold (COGS) – year 1</t>
+          <t>Cost of goods sold (COGS): year 1</t>
+        </is>
+      </c>
+      <c r="B35" s="135" t="inlineStr">
+        <is>
+          <t>Moves with revenue when gross margin stays flat.</t>
         </is>
       </c>
       <c r="F35" s="42">
@@ -2478,7 +2591,7 @@
     <row r="36">
       <c r="A36" s="41" t="inlineStr">
         <is>
-          <t>Cost of goods sold (COGS) – year 2</t>
+          <t>Cost of goods sold (COGS): year 2</t>
         </is>
       </c>
       <c r="F36" s="42">
@@ -2497,7 +2610,7 @@
     <row r="37">
       <c r="A37" s="41" t="inlineStr">
         <is>
-          <t>Cost of goods sold (COGS) – year 3</t>
+          <t>Cost of goods sold (COGS): year 3</t>
         </is>
       </c>
       <c r="F37" s="42">
@@ -2516,7 +2629,7 @@
     <row r="38">
       <c r="A38" s="41" t="inlineStr">
         <is>
-          <t>Cost of goods sold (COGS) – year 4</t>
+          <t>Cost of goods sold (COGS): year 4</t>
         </is>
       </c>
       <c r="F38" s="42">
@@ -2535,7 +2648,7 @@
     <row r="39">
       <c r="A39" s="41" t="inlineStr">
         <is>
-          <t>Cost of goods sold (COGS) – year 5</t>
+          <t>Cost of goods sold (COGS): year 5</t>
         </is>
       </c>
       <c r="F39" s="42">
@@ -2554,7 +2667,12 @@
     <row r="40">
       <c r="A40" s="41" t="inlineStr">
         <is>
-          <t>Clean EBIT margin – year 1</t>
+          <t>Clean EBIT margin: year 1</t>
+        </is>
+      </c>
+      <c r="B40" s="135" t="inlineStr">
+        <is>
+          <t>Linearly ramps from run-rate toward terminal margin.</t>
         </is>
       </c>
       <c r="F40" s="43">
@@ -2573,7 +2691,7 @@
     <row r="41">
       <c r="A41" s="41" t="inlineStr">
         <is>
-          <t>Clean EBIT margin – year 2</t>
+          <t>Clean EBIT margin: year 2</t>
         </is>
       </c>
       <c r="F41" s="43">
@@ -2592,7 +2710,7 @@
     <row r="42">
       <c r="A42" s="41" t="inlineStr">
         <is>
-          <t>Clean EBIT margin – year 3</t>
+          <t>Clean EBIT margin: year 3</t>
         </is>
       </c>
       <c r="F42" s="43">
@@ -2611,7 +2729,7 @@
     <row r="43">
       <c r="A43" s="41" t="inlineStr">
         <is>
-          <t>Clean EBIT margin – year 4</t>
+          <t>Clean EBIT margin: year 4</t>
         </is>
       </c>
       <c r="F43" s="43">
@@ -2630,7 +2748,7 @@
     <row r="44">
       <c r="A44" s="41" t="inlineStr">
         <is>
-          <t>Clean EBIT margin – year 5</t>
+          <t>Clean EBIT margin: year 5</t>
         </is>
       </c>
       <c r="F44" s="43">
@@ -2649,7 +2767,12 @@
     <row r="45">
       <c r="A45" s="41" t="inlineStr">
         <is>
-          <t>EBIT – year 1</t>
+          <t>EBIT: year 1</t>
+        </is>
+      </c>
+      <c r="B45" s="135" t="inlineStr">
+        <is>
+          <t>Revenue times margin: year one adds tariff refund.</t>
         </is>
       </c>
       <c r="F45" s="42">
@@ -2668,7 +2791,7 @@
     <row r="46">
       <c r="A46" s="41" t="inlineStr">
         <is>
-          <t>EBIT – year 2</t>
+          <t>EBIT: year 2</t>
         </is>
       </c>
       <c r="F46" s="42">
@@ -2687,7 +2810,7 @@
     <row r="47">
       <c r="A47" s="41" t="inlineStr">
         <is>
-          <t>EBIT – year 3</t>
+          <t>EBIT: year 3</t>
         </is>
       </c>
       <c r="F47" s="42">
@@ -2706,7 +2829,7 @@
     <row r="48">
       <c r="A48" s="41" t="inlineStr">
         <is>
-          <t>EBIT – year 4</t>
+          <t>EBIT: year 4</t>
         </is>
       </c>
       <c r="F48" s="42">
@@ -2725,7 +2848,7 @@
     <row r="49">
       <c r="A49" s="41" t="inlineStr">
         <is>
-          <t>EBIT – year 5</t>
+          <t>EBIT: year 5</t>
         </is>
       </c>
       <c r="F49" s="42">
@@ -2744,7 +2867,12 @@
     <row r="50">
       <c r="A50" s="41" t="inlineStr">
         <is>
-          <t>NOPAT – year 1</t>
+          <t>NOPAT: year 1</t>
+        </is>
+      </c>
+      <c r="B50" s="135" t="inlineStr">
+        <is>
+          <t>EBIT taxed at flat cash rate each year.</t>
         </is>
       </c>
       <c r="F50" s="42">
@@ -2763,7 +2891,7 @@
     <row r="51">
       <c r="A51" s="41" t="inlineStr">
         <is>
-          <t>NOPAT – year 2</t>
+          <t>NOPAT: year 2</t>
         </is>
       </c>
       <c r="F51" s="42">
@@ -2782,7 +2910,7 @@
     <row r="52">
       <c r="A52" s="41" t="inlineStr">
         <is>
-          <t>NOPAT – year 3</t>
+          <t>NOPAT: year 3</t>
         </is>
       </c>
       <c r="F52" s="42">
@@ -2801,7 +2929,7 @@
     <row r="53">
       <c r="A53" s="41" t="inlineStr">
         <is>
-          <t>NOPAT – year 4</t>
+          <t>NOPAT: year 4</t>
         </is>
       </c>
       <c r="F53" s="42">
@@ -2820,7 +2948,7 @@
     <row r="54">
       <c r="A54" s="41" t="inlineStr">
         <is>
-          <t>NOPAT – year 5</t>
+          <t>NOPAT: year 5</t>
         </is>
       </c>
       <c r="F54" s="42">
@@ -2839,7 +2967,12 @@
     <row r="55">
       <c r="A55" s="41" t="inlineStr">
         <is>
-          <t>D&amp;A – year 1</t>
+          <t>D&amp;A: year 1</t>
+        </is>
+      </c>
+      <c r="B55" s="135" t="inlineStr">
+        <is>
+          <t>Scales upward with revenue at fixed percentage annually.</t>
         </is>
       </c>
       <c r="F55" s="42">
@@ -2858,7 +2991,7 @@
     <row r="56">
       <c r="A56" s="41" t="inlineStr">
         <is>
-          <t>D&amp;A – year 2</t>
+          <t>D&amp;A: year 2</t>
         </is>
       </c>
       <c r="F56" s="42">
@@ -2877,7 +3010,7 @@
     <row r="57">
       <c r="A57" s="41" t="inlineStr">
         <is>
-          <t>D&amp;A – year 3</t>
+          <t>D&amp;A: year 3</t>
         </is>
       </c>
       <c r="F57" s="42">
@@ -2896,7 +3029,7 @@
     <row r="58">
       <c r="A58" s="41" t="inlineStr">
         <is>
-          <t>D&amp;A – year 4</t>
+          <t>D&amp;A: year 4</t>
         </is>
       </c>
       <c r="F58" s="42">
@@ -2915,7 +3048,7 @@
     <row r="59">
       <c r="A59" s="41" t="inlineStr">
         <is>
-          <t>D&amp;A – year 5</t>
+          <t>D&amp;A: year 5</t>
         </is>
       </c>
       <c r="F59" s="42">
@@ -2934,7 +3067,12 @@
     <row r="60">
       <c r="A60" s="41" t="inlineStr">
         <is>
-          <t>Capex – year 1</t>
+          <t>Capex: year 1</t>
+        </is>
+      </c>
+      <c r="B60" s="135" t="inlineStr">
+        <is>
+          <t>Scales upward with revenue at fixed percentage annually.</t>
         </is>
       </c>
       <c r="F60" s="42">
@@ -2953,7 +3091,7 @@
     <row r="61">
       <c r="A61" s="41" t="inlineStr">
         <is>
-          <t>Capex – year 2</t>
+          <t>Capex: year 2</t>
         </is>
       </c>
       <c r="F61" s="42">
@@ -2972,7 +3110,7 @@
     <row r="62">
       <c r="A62" s="41" t="inlineStr">
         <is>
-          <t>Capex – year 3</t>
+          <t>Capex: year 3</t>
         </is>
       </c>
       <c r="F62" s="42">
@@ -2991,7 +3129,7 @@
     <row r="63">
       <c r="A63" s="41" t="inlineStr">
         <is>
-          <t>Capex – year 4</t>
+          <t>Capex: year 4</t>
         </is>
       </c>
       <c r="F63" s="42">
@@ -3010,7 +3148,7 @@
     <row r="64">
       <c r="A64" s="41" t="inlineStr">
         <is>
-          <t>Capex – year 5</t>
+          <t>Capex: year 5</t>
         </is>
       </c>
       <c r="F64" s="42">
@@ -3029,7 +3167,12 @@
     <row r="65">
       <c r="A65" s="41" t="inlineStr">
         <is>
-          <t>DSO (days) – year 1</t>
+          <t>DSO (days): year 1</t>
+        </is>
+      </c>
+      <c r="B65" s="135" t="inlineStr">
+        <is>
+          <t>Held flat at six days every forecast year.</t>
         </is>
       </c>
       <c r="F65" s="44">
@@ -3048,7 +3191,7 @@
     <row r="66">
       <c r="A66" s="41" t="inlineStr">
         <is>
-          <t>DSO (days) – year 2</t>
+          <t>DSO (days): year 2</t>
         </is>
       </c>
       <c r="F66" s="44">
@@ -3067,7 +3210,7 @@
     <row r="67">
       <c r="A67" s="41" t="inlineStr">
         <is>
-          <t>DSO (days) – year 3</t>
+          <t>DSO (days): year 3</t>
         </is>
       </c>
       <c r="F67" s="44">
@@ -3086,7 +3229,7 @@
     <row r="68">
       <c r="A68" s="41" t="inlineStr">
         <is>
-          <t>DSO (days) – year 4</t>
+          <t>DSO (days): year 4</t>
         </is>
       </c>
       <c r="F68" s="44">
@@ -3105,7 +3248,7 @@
     <row r="69">
       <c r="A69" s="41" t="inlineStr">
         <is>
-          <t>DSO (days) – year 5</t>
+          <t>DSO (days): year 5</t>
         </is>
       </c>
       <c r="F69" s="44">
@@ -3124,7 +3267,12 @@
     <row r="70">
       <c r="A70" s="41" t="inlineStr">
         <is>
-          <t>Accounts receivable – year 1</t>
+          <t>Accounts receivable: year 1</t>
+        </is>
+      </c>
+      <c r="B70" s="135" t="inlineStr">
+        <is>
+          <t>Tracks revenue changes while collection days stay flat.</t>
         </is>
       </c>
       <c r="F70" s="42">
@@ -3143,7 +3291,7 @@
     <row r="71">
       <c r="A71" s="41" t="inlineStr">
         <is>
-          <t>Accounts receivable – year 2</t>
+          <t>Accounts receivable: year 2</t>
         </is>
       </c>
       <c r="F71" s="42">
@@ -3162,7 +3310,7 @@
     <row r="72">
       <c r="A72" s="41" t="inlineStr">
         <is>
-          <t>Accounts receivable – year 3</t>
+          <t>Accounts receivable: year 3</t>
         </is>
       </c>
       <c r="F72" s="42">
@@ -3181,7 +3329,7 @@
     <row r="73">
       <c r="A73" s="41" t="inlineStr">
         <is>
-          <t>Accounts receivable – year 4</t>
+          <t>Accounts receivable: year 4</t>
         </is>
       </c>
       <c r="F73" s="42">
@@ -3200,7 +3348,7 @@
     <row r="74">
       <c r="A74" s="41" t="inlineStr">
         <is>
-          <t>Accounts receivable – year 5</t>
+          <t>Accounts receivable: year 5</t>
         </is>
       </c>
       <c r="F74" s="42">
@@ -3219,7 +3367,12 @@
     <row r="75">
       <c r="A75" s="41" t="inlineStr">
         <is>
-          <t>DIO (days) – year 1</t>
+          <t>DIO (days): year 1</t>
+        </is>
+      </c>
+      <c r="B75" s="135" t="inlineStr">
+        <is>
+          <t>Falls one day per year across five years.</t>
         </is>
       </c>
       <c r="F75" s="44">
@@ -3238,7 +3391,7 @@
     <row r="76">
       <c r="A76" s="41" t="inlineStr">
         <is>
-          <t>DIO (days) – year 2</t>
+          <t>DIO (days): year 2</t>
         </is>
       </c>
       <c r="F76" s="44">
@@ -3257,7 +3410,7 @@
     <row r="77">
       <c r="A77" s="41" t="inlineStr">
         <is>
-          <t>DIO (days) – year 3</t>
+          <t>DIO (days): year 3</t>
         </is>
       </c>
       <c r="F77" s="44">
@@ -3276,7 +3429,7 @@
     <row r="78">
       <c r="A78" s="41" t="inlineStr">
         <is>
-          <t>DIO (days) – year 4</t>
+          <t>DIO (days): year 4</t>
         </is>
       </c>
       <c r="F78" s="44">
@@ -3295,7 +3448,7 @@
     <row r="79">
       <c r="A79" s="41" t="inlineStr">
         <is>
-          <t>DIO (days) – year 5</t>
+          <t>DIO (days): year 5</t>
         </is>
       </c>
       <c r="F79" s="44">
@@ -3314,7 +3467,12 @@
     <row r="80">
       <c r="A80" s="41" t="inlineStr">
         <is>
-          <t>Inventories – year 1</t>
+          <t>Inventories: year 1</t>
+        </is>
+      </c>
+      <c r="B80" s="135" t="inlineStr">
+        <is>
+          <t>Declines with DIO days: grows with rising COGS.</t>
         </is>
       </c>
       <c r="F80" s="42">
@@ -3333,7 +3491,7 @@
     <row r="81">
       <c r="A81" s="41" t="inlineStr">
         <is>
-          <t>Inventories – year 2</t>
+          <t>Inventories: year 2</t>
         </is>
       </c>
       <c r="F81" s="42">
@@ -3352,7 +3510,7 @@
     <row r="82">
       <c r="A82" s="41" t="inlineStr">
         <is>
-          <t>Inventories – year 3</t>
+          <t>Inventories: year 3</t>
         </is>
       </c>
       <c r="F82" s="42">
@@ -3371,7 +3529,7 @@
     <row r="83">
       <c r="A83" s="41" t="inlineStr">
         <is>
-          <t>Inventories – year 4</t>
+          <t>Inventories: year 4</t>
         </is>
       </c>
       <c r="F83" s="42">
@@ -3390,7 +3548,7 @@
     <row r="84">
       <c r="A84" s="41" t="inlineStr">
         <is>
-          <t>Inventories – year 5</t>
+          <t>Inventories: year 5</t>
         </is>
       </c>
       <c r="F84" s="42">
@@ -3409,7 +3567,12 @@
     <row r="85">
       <c r="A85" s="41" t="inlineStr">
         <is>
-          <t>DPO (days) – year 1</t>
+          <t>DPO (days): year 1</t>
+        </is>
+      </c>
+      <c r="B85" s="135" t="inlineStr">
+        <is>
+          <t>Held flat at twenty-five days every year.</t>
         </is>
       </c>
       <c r="F85" s="44">
@@ -3428,7 +3591,7 @@
     <row r="86">
       <c r="A86" s="41" t="inlineStr">
         <is>
-          <t>DPO (days) – year 2</t>
+          <t>DPO (days): year 2</t>
         </is>
       </c>
       <c r="F86" s="44">
@@ -3447,7 +3610,7 @@
     <row r="87">
       <c r="A87" s="41" t="inlineStr">
         <is>
-          <t>DPO (days) – year 3</t>
+          <t>DPO (days): year 3</t>
         </is>
       </c>
       <c r="F87" s="44">
@@ -3466,7 +3629,7 @@
     <row r="88">
       <c r="A88" s="41" t="inlineStr">
         <is>
-          <t>DPO (days) – year 4</t>
+          <t>DPO (days): year 4</t>
         </is>
       </c>
       <c r="F88" s="44">
@@ -3485,7 +3648,7 @@
     <row r="89">
       <c r="A89" s="41" t="inlineStr">
         <is>
-          <t>DPO (days) – year 5</t>
+          <t>DPO (days): year 5</t>
         </is>
       </c>
       <c r="F89" s="44">
@@ -3504,7 +3667,12 @@
     <row r="90">
       <c r="A90" s="41" t="inlineStr">
         <is>
-          <t>Accounts payable – year 1</t>
+          <t>Accounts payable: year 1</t>
+        </is>
+      </c>
+      <c r="B90" s="135" t="inlineStr">
+        <is>
+          <t>Grows with COGS while payment days remain flat.</t>
         </is>
       </c>
       <c r="F90" s="42">
@@ -3523,7 +3691,7 @@
     <row r="91">
       <c r="A91" s="41" t="inlineStr">
         <is>
-          <t>Accounts payable – year 2</t>
+          <t>Accounts payable: year 2</t>
         </is>
       </c>
       <c r="F91" s="42">
@@ -3542,7 +3710,7 @@
     <row r="92">
       <c r="A92" s="41" t="inlineStr">
         <is>
-          <t>Accounts payable – year 3</t>
+          <t>Accounts payable: year 3</t>
         </is>
       </c>
       <c r="F92" s="42">
@@ -3561,7 +3729,7 @@
     <row r="93">
       <c r="A93" s="41" t="inlineStr">
         <is>
-          <t>Accounts payable – year 4</t>
+          <t>Accounts payable: year 4</t>
         </is>
       </c>
       <c r="F93" s="42">
@@ -3580,7 +3748,7 @@
     <row r="94">
       <c r="A94" s="41" t="inlineStr">
         <is>
-          <t>Accounts payable – year 5</t>
+          <t>Accounts payable: year 5</t>
         </is>
       </c>
       <c r="F94" s="42">
@@ -3599,7 +3767,12 @@
     <row r="95">
       <c r="A95" s="41" t="inlineStr">
         <is>
-          <t>Prepaid expenses (other current assets) – year 1</t>
+          <t>Prepaid expenses (other current assets): year 1</t>
+        </is>
+      </c>
+      <c r="B95" s="135" t="inlineStr">
+        <is>
+          <t>Grows at flat percent of revenue yearly.</t>
         </is>
       </c>
       <c r="F95" s="42">
@@ -3618,7 +3791,7 @@
     <row r="96">
       <c r="A96" s="41" t="inlineStr">
         <is>
-          <t>Prepaid expenses (other current assets) – year 2</t>
+          <t>Prepaid expenses (other current assets): year 2</t>
         </is>
       </c>
       <c r="F96" s="42">
@@ -3637,7 +3810,7 @@
     <row r="97">
       <c r="A97" s="41" t="inlineStr">
         <is>
-          <t>Prepaid expenses (other current assets) – year 3</t>
+          <t>Prepaid expenses (other current assets): year 3</t>
         </is>
       </c>
       <c r="F97" s="42">
@@ -3656,7 +3829,7 @@
     <row r="98">
       <c r="A98" s="41" t="inlineStr">
         <is>
-          <t>Prepaid expenses (other current assets) – year 4</t>
+          <t>Prepaid expenses (other current assets): year 4</t>
         </is>
       </c>
       <c r="F98" s="42">
@@ -3675,7 +3848,7 @@
     <row r="99">
       <c r="A99" s="41" t="inlineStr">
         <is>
-          <t>Prepaid expenses (other current assets) – year 5</t>
+          <t>Prepaid expenses (other current assets): year 5</t>
         </is>
       </c>
       <c r="F99" s="42">
@@ -3694,7 +3867,12 @@
     <row r="100">
       <c r="A100" s="41" t="inlineStr">
         <is>
-          <t>Accrued liabilities – year 1</t>
+          <t>Accrued liabilities: year 1</t>
+        </is>
+      </c>
+      <c r="B100" s="135" t="inlineStr">
+        <is>
+          <t>Grows at flat percent of revenue every year.</t>
         </is>
       </c>
       <c r="F100" s="42">
@@ -3713,7 +3891,7 @@
     <row r="101">
       <c r="A101" s="41" t="inlineStr">
         <is>
-          <t>Accrued liabilities – year 2</t>
+          <t>Accrued liabilities: year 2</t>
         </is>
       </c>
       <c r="F101" s="42">
@@ -3732,7 +3910,7 @@
     <row r="102">
       <c r="A102" s="41" t="inlineStr">
         <is>
-          <t>Accrued liabilities – year 3</t>
+          <t>Accrued liabilities: year 3</t>
         </is>
       </c>
       <c r="F102" s="42">
@@ -3751,7 +3929,7 @@
     <row r="103">
       <c r="A103" s="41" t="inlineStr">
         <is>
-          <t>Accrued liabilities – year 4</t>
+          <t>Accrued liabilities: year 4</t>
         </is>
       </c>
       <c r="F103" s="42">
@@ -3770,7 +3948,7 @@
     <row r="104">
       <c r="A104" s="41" t="inlineStr">
         <is>
-          <t>Accrued liabilities – year 5</t>
+          <t>Accrued liabilities: year 5</t>
         </is>
       </c>
       <c r="F104" s="42">
@@ -3789,7 +3967,12 @@
     <row r="105">
       <c r="A105" s="41" t="inlineStr">
         <is>
-          <t>Current operating assets (AR + inv + prepaids) – year 1</t>
+          <t>Current operating assets (AR + inv + prepaids): year 1</t>
+        </is>
+      </c>
+      <c r="B105" s="135" t="inlineStr">
+        <is>
+          <t>Rises as receivables, inventory, prepaids expand.</t>
         </is>
       </c>
       <c r="F105" s="42">
@@ -3808,7 +3991,7 @@
     <row r="106">
       <c r="A106" s="41" t="inlineStr">
         <is>
-          <t>Current operating assets (AR + inv + prepaids) – year 2</t>
+          <t>Current operating assets (AR + inv + prepaids): year 2</t>
         </is>
       </c>
       <c r="F106" s="42">
@@ -3827,7 +4010,7 @@
     <row r="107">
       <c r="A107" s="41" t="inlineStr">
         <is>
-          <t>Current operating assets (AR + inv + prepaids) – year 3</t>
+          <t>Current operating assets (AR + inv + prepaids): year 3</t>
         </is>
       </c>
       <c r="F107" s="42">
@@ -3846,7 +4029,7 @@
     <row r="108">
       <c r="A108" s="41" t="inlineStr">
         <is>
-          <t>Current operating assets (AR + inv + prepaids) – year 4</t>
+          <t>Current operating assets (AR + inv + prepaids): year 4</t>
         </is>
       </c>
       <c r="F108" s="42">
@@ -3865,7 +4048,7 @@
     <row r="109">
       <c r="A109" s="41" t="inlineStr">
         <is>
-          <t>Current operating assets (AR + inv + prepaids) – year 5</t>
+          <t>Current operating assets (AR + inv + prepaids): year 5</t>
         </is>
       </c>
       <c r="F109" s="42">
@@ -3884,7 +4067,12 @@
     <row r="110">
       <c r="A110" s="41" t="inlineStr">
         <is>
-          <t>Current operating liabilities (AP + accruals) – year 1</t>
+          <t>Current operating liabilities (AP + accruals): year 1</t>
+        </is>
+      </c>
+      <c r="B110" s="135" t="inlineStr">
+        <is>
+          <t>Rises as payables and accruals grow with sales.</t>
         </is>
       </c>
       <c r="F110" s="42">
@@ -3903,7 +4091,7 @@
     <row r="111">
       <c r="A111" s="41" t="inlineStr">
         <is>
-          <t>Current operating liabilities (AP + accruals) – year 2</t>
+          <t>Current operating liabilities (AP + accruals): year 2</t>
         </is>
       </c>
       <c r="F111" s="42">
@@ -3922,7 +4110,7 @@
     <row r="112">
       <c r="A112" s="41" t="inlineStr">
         <is>
-          <t>Current operating liabilities (AP + accruals) – year 3</t>
+          <t>Current operating liabilities (AP + accruals): year 3</t>
         </is>
       </c>
       <c r="F112" s="42">
@@ -3941,7 +4129,7 @@
     <row r="113">
       <c r="A113" s="41" t="inlineStr">
         <is>
-          <t>Current operating liabilities (AP + accruals) – year 4</t>
+          <t>Current operating liabilities (AP + accruals): year 4</t>
         </is>
       </c>
       <c r="F113" s="42">
@@ -3960,7 +4148,7 @@
     <row r="114">
       <c r="A114" s="41" t="inlineStr">
         <is>
-          <t>Current operating liabilities (AP + accruals) – year 5</t>
+          <t>Current operating liabilities (AP + accruals): year 5</t>
         </is>
       </c>
       <c r="F114" s="42">
@@ -3979,7 +4167,12 @@
     <row r="115">
       <c r="A115" s="41" t="inlineStr">
         <is>
-          <t>Net working capital – year 1</t>
+          <t>Net working capital: year 1</t>
+        </is>
+      </c>
+      <c r="B115" s="135" t="inlineStr">
+        <is>
+          <t>Operating assets minus liabilities: level shifts yearly.</t>
         </is>
       </c>
       <c r="F115" s="42">
@@ -3998,7 +4191,7 @@
     <row r="116">
       <c r="A116" s="41" t="inlineStr">
         <is>
-          <t>Net working capital – year 2</t>
+          <t>Net working capital: year 2</t>
         </is>
       </c>
       <c r="F116" s="42">
@@ -4017,7 +4210,7 @@
     <row r="117">
       <c r="A117" s="41" t="inlineStr">
         <is>
-          <t>Net working capital – year 3</t>
+          <t>Net working capital: year 3</t>
         </is>
       </c>
       <c r="F117" s="42">
@@ -4036,7 +4229,7 @@
     <row r="118">
       <c r="A118" s="41" t="inlineStr">
         <is>
-          <t>Net working capital – year 4</t>
+          <t>Net working capital: year 4</t>
         </is>
       </c>
       <c r="F118" s="42">
@@ -4055,7 +4248,7 @@
     <row r="119">
       <c r="A119" s="41" t="inlineStr">
         <is>
-          <t>Net working capital – year 5</t>
+          <t>Net working capital: year 5</t>
         </is>
       </c>
       <c r="F119" s="42">
@@ -4074,7 +4267,12 @@
     <row r="120">
       <c r="A120" s="41" t="inlineStr">
         <is>
-          <t>ΔNWC (prior yr − current yr) – year 1</t>
+          <t>ΔNWC (prior yr: prior yr minus current yr): year 1</t>
+        </is>
+      </c>
+      <c r="B120" s="135" t="inlineStr">
+        <is>
+          <t>Prior minus current NWC: positive releases cash.</t>
         </is>
       </c>
       <c r="F120" s="42">
@@ -4093,7 +4291,7 @@
     <row r="121">
       <c r="A121" s="41" t="inlineStr">
         <is>
-          <t>ΔNWC (prior yr − current yr) – year 2</t>
+          <t>ΔNWC (prior yr: prior yr minus current yr): year 2</t>
         </is>
       </c>
       <c r="F121" s="42">
@@ -4112,7 +4310,7 @@
     <row r="122">
       <c r="A122" s="41" t="inlineStr">
         <is>
-          <t>ΔNWC (prior yr − current yr) – year 3</t>
+          <t>ΔNWC (prior yr: prior yr minus current yr): year 3</t>
         </is>
       </c>
       <c r="F122" s="42">
@@ -4131,7 +4329,7 @@
     <row r="123">
       <c r="A123" s="41" t="inlineStr">
         <is>
-          <t>ΔNWC (prior yr − current yr) – year 4</t>
+          <t>ΔNWC (prior yr: prior yr minus current yr): year 4</t>
         </is>
       </c>
       <c r="F123" s="42">
@@ -4150,7 +4348,7 @@
     <row r="124">
       <c r="A124" s="41" t="inlineStr">
         <is>
-          <t>ΔNWC (prior yr − current yr) – year 5</t>
+          <t>ΔNWC (prior yr: prior yr minus current yr): year 5</t>
         </is>
       </c>
       <c r="F124" s="42">
@@ -4169,7 +4367,12 @@
     <row r="125">
       <c r="A125" s="41" t="inlineStr">
         <is>
-          <t>Unlevered FCF – year 1</t>
+          <t>Unlevered FCF: year 1</t>
+        </is>
+      </c>
+      <c r="B125" s="135" t="inlineStr">
+        <is>
+          <t>NOPAT plus depreciation minus capex plus working capital.</t>
         </is>
       </c>
       <c r="F125" s="42">
@@ -4188,7 +4391,7 @@
     <row r="126">
       <c r="A126" s="41" t="inlineStr">
         <is>
-          <t>Unlevered FCF – year 2</t>
+          <t>Unlevered FCF: year 2</t>
         </is>
       </c>
       <c r="F126" s="42">
@@ -4207,7 +4410,7 @@
     <row r="127">
       <c r="A127" s="41" t="inlineStr">
         <is>
-          <t>Unlevered FCF – year 3</t>
+          <t>Unlevered FCF: year 3</t>
         </is>
       </c>
       <c r="F127" s="42">
@@ -4226,7 +4429,7 @@
     <row r="128">
       <c r="A128" s="41" t="inlineStr">
         <is>
-          <t>Unlevered FCF – year 4</t>
+          <t>Unlevered FCF: year 4</t>
         </is>
       </c>
       <c r="F128" s="42">
@@ -4245,7 +4448,7 @@
     <row r="129">
       <c r="A129" s="41" t="inlineStr">
         <is>
-          <t>Unlevered FCF – year 5</t>
+          <t>Unlevered FCF: year 5</t>
         </is>
       </c>
       <c r="F129" s="42">
@@ -4261,6 +4464,7 @@
         <v/>
       </c>
     </row>
+    <row r="130"/>
     <row r="131">
       <c r="A131" s="23" t="inlineStr">
         <is>
@@ -4318,6 +4522,7 @@
         <v/>
       </c>
     </row>
+    <row r="134"/>
     <row r="135">
       <c r="A135" s="26" t="inlineStr">
         <is>
@@ -4325,6 +4530,7 @@
         </is>
       </c>
     </row>
+    <row r="136"/>
     <row r="137">
       <c r="A137" s="14" t="inlineStr">
         <is>
@@ -4335,7 +4541,7 @@
     <row r="138">
       <c r="A138" s="41" t="inlineStr">
         <is>
-          <t>Other income – year 1</t>
+          <t>Other income: year 1</t>
         </is>
       </c>
       <c r="F138" s="42" t="n">
@@ -4351,7 +4557,7 @@
     <row r="139">
       <c r="A139" s="41" t="inlineStr">
         <is>
-          <t>Other income – year 2</t>
+          <t>Other income: year 2</t>
         </is>
       </c>
       <c r="F139" s="42" t="n">
@@ -4367,7 +4573,7 @@
     <row r="140">
       <c r="A140" s="41" t="inlineStr">
         <is>
-          <t>Other income – year 3</t>
+          <t>Other income: year 3</t>
         </is>
       </c>
       <c r="F140" s="42" t="n">
@@ -4383,7 +4589,7 @@
     <row r="141">
       <c r="A141" s="41" t="inlineStr">
         <is>
-          <t>Other income – year 4</t>
+          <t>Other income: year 4</t>
         </is>
       </c>
       <c r="F141" s="42" t="n">
@@ -4399,7 +4605,7 @@
     <row r="142">
       <c r="A142" s="41" t="inlineStr">
         <is>
-          <t>Other income – year 5</t>
+          <t>Other income: year 5</t>
         </is>
       </c>
       <c r="F142" s="42" t="n">
@@ -4415,7 +4621,7 @@
     <row r="143">
       <c r="A143" s="41" t="inlineStr">
         <is>
-          <t>Net income – year 1</t>
+          <t>Net income: year 1</t>
         </is>
       </c>
       <c r="F143" s="42">
@@ -4434,7 +4640,7 @@
     <row r="144">
       <c r="A144" s="41" t="inlineStr">
         <is>
-          <t>Net income – year 2</t>
+          <t>Net income: year 2</t>
         </is>
       </c>
       <c r="F144" s="42">
@@ -4453,7 +4659,7 @@
     <row r="145">
       <c r="A145" s="41" t="inlineStr">
         <is>
-          <t>Net income – year 3</t>
+          <t>Net income: year 3</t>
         </is>
       </c>
       <c r="F145" s="42">
@@ -4472,7 +4678,7 @@
     <row r="146">
       <c r="A146" s="41" t="inlineStr">
         <is>
-          <t>Net income – year 4</t>
+          <t>Net income: year 4</t>
         </is>
       </c>
       <c r="F146" s="42">
@@ -4491,7 +4697,7 @@
     <row r="147">
       <c r="A147" s="41" t="inlineStr">
         <is>
-          <t>Net income – year 5</t>
+          <t>Net income: year 5</t>
         </is>
       </c>
       <c r="F147" s="42">
@@ -4510,7 +4716,7 @@
     <row r="148">
       <c r="A148" s="41" t="inlineStr">
         <is>
-          <t>Cash from operations – year 1</t>
+          <t>Cash from operations: year 1</t>
         </is>
       </c>
       <c r="F148" s="42">
@@ -4529,7 +4735,7 @@
     <row r="149">
       <c r="A149" s="41" t="inlineStr">
         <is>
-          <t>Cash from operations – year 2</t>
+          <t>Cash from operations: year 2</t>
         </is>
       </c>
       <c r="F149" s="42">
@@ -4548,7 +4754,7 @@
     <row r="150">
       <c r="A150" s="41" t="inlineStr">
         <is>
-          <t>Cash from operations – year 3</t>
+          <t>Cash from operations: year 3</t>
         </is>
       </c>
       <c r="F150" s="42">
@@ -4567,7 +4773,7 @@
     <row r="151">
       <c r="A151" s="41" t="inlineStr">
         <is>
-          <t>Cash from operations – year 4</t>
+          <t>Cash from operations: year 4</t>
         </is>
       </c>
       <c r="F151" s="42">
@@ -4586,7 +4792,7 @@
     <row r="152">
       <c r="A152" s="41" t="inlineStr">
         <is>
-          <t>Cash from operations – year 5</t>
+          <t>Cash from operations: year 5</t>
         </is>
       </c>
       <c r="F152" s="42">
@@ -4605,7 +4811,7 @@
     <row r="153">
       <c r="A153" s="41" t="inlineStr">
         <is>
-          <t>Free cash flow (CFS) – year 1</t>
+          <t>Free cash flow (CFS): year 1</t>
         </is>
       </c>
       <c r="F153" s="42">
@@ -4624,7 +4830,7 @@
     <row r="154">
       <c r="A154" s="41" t="inlineStr">
         <is>
-          <t>Free cash flow (CFS) – year 2</t>
+          <t>Free cash flow (CFS): year 2</t>
         </is>
       </c>
       <c r="F154" s="42">
@@ -4643,7 +4849,7 @@
     <row r="155">
       <c r="A155" s="41" t="inlineStr">
         <is>
-          <t>Free cash flow (CFS) – year 3</t>
+          <t>Free cash flow (CFS): year 3</t>
         </is>
       </c>
       <c r="F155" s="42">
@@ -4662,7 +4868,7 @@
     <row r="156">
       <c r="A156" s="41" t="inlineStr">
         <is>
-          <t>Free cash flow (CFS) – year 4</t>
+          <t>Free cash flow (CFS): year 4</t>
         </is>
       </c>
       <c r="F156" s="42">
@@ -4681,7 +4887,7 @@
     <row r="157">
       <c r="A157" s="41" t="inlineStr">
         <is>
-          <t>Free cash flow (CFS) – year 5</t>
+          <t>Free cash flow (CFS): year 5</t>
         </is>
       </c>
       <c r="F157" s="42">
@@ -4700,7 +4906,7 @@
     <row r="158">
       <c r="A158" s="41" t="inlineStr">
         <is>
-          <t>Share repurchases – year 1</t>
+          <t>Share repurchases: year 1</t>
         </is>
       </c>
       <c r="F158" s="42">
@@ -4719,7 +4925,7 @@
     <row r="159">
       <c r="A159" s="41" t="inlineStr">
         <is>
-          <t>Share repurchases – year 2</t>
+          <t>Share repurchases: year 2</t>
         </is>
       </c>
       <c r="F159" s="42">
@@ -4738,7 +4944,7 @@
     <row r="160">
       <c r="A160" s="41" t="inlineStr">
         <is>
-          <t>Share repurchases – year 3</t>
+          <t>Share repurchases: year 3</t>
         </is>
       </c>
       <c r="F160" s="42">
@@ -4757,7 +4963,7 @@
     <row r="161">
       <c r="A161" s="41" t="inlineStr">
         <is>
-          <t>Share repurchases – year 4</t>
+          <t>Share repurchases: year 4</t>
         </is>
       </c>
       <c r="F161" s="42">
@@ -4776,7 +4982,7 @@
     <row r="162">
       <c r="A162" s="41" t="inlineStr">
         <is>
-          <t>Share repurchases – year 5</t>
+          <t>Share repurchases: year 5</t>
         </is>
       </c>
       <c r="F162" s="42">
@@ -4795,7 +5001,7 @@
     <row r="163">
       <c r="A163" s="41" t="inlineStr">
         <is>
-          <t>Cash &amp; equivalents – year 1</t>
+          <t>Cash &amp; equivalents: year 1</t>
         </is>
       </c>
       <c r="F163" s="42">
@@ -4814,7 +5020,7 @@
     <row r="164">
       <c r="A164" s="41" t="inlineStr">
         <is>
-          <t>Cash &amp; equivalents – year 2</t>
+          <t>Cash &amp; equivalents: year 2</t>
         </is>
       </c>
       <c r="F164" s="42">
@@ -4833,7 +5039,7 @@
     <row r="165">
       <c r="A165" s="41" t="inlineStr">
         <is>
-          <t>Cash &amp; equivalents – year 3</t>
+          <t>Cash &amp; equivalents: year 3</t>
         </is>
       </c>
       <c r="F165" s="42">
@@ -4852,7 +5058,7 @@
     <row r="166">
       <c r="A166" s="41" t="inlineStr">
         <is>
-          <t>Cash &amp; equivalents – year 4</t>
+          <t>Cash &amp; equivalents: year 4</t>
         </is>
       </c>
       <c r="F166" s="42">
@@ -4871,7 +5077,7 @@
     <row r="167">
       <c r="A167" s="41" t="inlineStr">
         <is>
-          <t>Cash &amp; equivalents – year 5</t>
+          <t>Cash &amp; equivalents: year 5</t>
         </is>
       </c>
       <c r="F167" s="42">
@@ -4890,7 +5096,7 @@
     <row r="168">
       <c r="A168" s="41" t="inlineStr">
         <is>
-          <t>Total assets – year 1</t>
+          <t>Total assets: year 1</t>
         </is>
       </c>
       <c r="F168" s="42">
@@ -4909,7 +5115,7 @@
     <row r="169">
       <c r="A169" s="41" t="inlineStr">
         <is>
-          <t>Total assets – year 2</t>
+          <t>Total assets: year 2</t>
         </is>
       </c>
       <c r="F169" s="42">
@@ -4928,7 +5134,7 @@
     <row r="170">
       <c r="A170" s="41" t="inlineStr">
         <is>
-          <t>Total assets – year 3</t>
+          <t>Total assets: year 3</t>
         </is>
       </c>
       <c r="F170" s="42">
@@ -4947,7 +5153,7 @@
     <row r="171">
       <c r="A171" s="41" t="inlineStr">
         <is>
-          <t>Total assets – year 4</t>
+          <t>Total assets: year 4</t>
         </is>
       </c>
       <c r="F171" s="42">
@@ -4966,7 +5172,7 @@
     <row r="172">
       <c r="A172" s="41" t="inlineStr">
         <is>
-          <t>Total assets – year 5</t>
+          <t>Total assets: year 5</t>
         </is>
       </c>
       <c r="F172" s="42">
@@ -4985,7 +5191,7 @@
     <row r="173">
       <c r="A173" s="41" t="inlineStr">
         <is>
-          <t>Total liabilities – year 1</t>
+          <t>Total liabilities: year 1</t>
         </is>
       </c>
       <c r="F173" s="42">
@@ -5004,7 +5210,7 @@
     <row r="174">
       <c r="A174" s="41" t="inlineStr">
         <is>
-          <t>Total liabilities – year 2</t>
+          <t>Total liabilities: year 2</t>
         </is>
       </c>
       <c r="F174" s="42">
@@ -5023,7 +5229,7 @@
     <row r="175">
       <c r="A175" s="41" t="inlineStr">
         <is>
-          <t>Total liabilities – year 3</t>
+          <t>Total liabilities: year 3</t>
         </is>
       </c>
       <c r="F175" s="42">
@@ -5042,7 +5248,7 @@
     <row r="176">
       <c r="A176" s="41" t="inlineStr">
         <is>
-          <t>Total liabilities – year 4</t>
+          <t>Total liabilities: year 4</t>
         </is>
       </c>
       <c r="F176" s="42">
@@ -5061,7 +5267,7 @@
     <row r="177">
       <c r="A177" s="41" t="inlineStr">
         <is>
-          <t>Total liabilities – year 5</t>
+          <t>Total liabilities: year 5</t>
         </is>
       </c>
       <c r="F177" s="42">
@@ -5080,7 +5286,7 @@
     <row r="178">
       <c r="A178" s="41" t="inlineStr">
         <is>
-          <t>Total equity – year 1</t>
+          <t>Total equity: year 1</t>
         </is>
       </c>
       <c r="F178" s="42">
@@ -5099,7 +5305,7 @@
     <row r="179">
       <c r="A179" s="41" t="inlineStr">
         <is>
-          <t>Total equity – year 2</t>
+          <t>Total equity: year 2</t>
         </is>
       </c>
       <c r="F179" s="42">
@@ -5118,7 +5324,7 @@
     <row r="180">
       <c r="A180" s="41" t="inlineStr">
         <is>
-          <t>Total equity – year 3</t>
+          <t>Total equity: year 3</t>
         </is>
       </c>
       <c r="F180" s="42">
@@ -5137,7 +5343,7 @@
     <row r="181">
       <c r="A181" s="41" t="inlineStr">
         <is>
-          <t>Total equity – year 4</t>
+          <t>Total equity: year 4</t>
         </is>
       </c>
       <c r="F181" s="42">
@@ -5156,7 +5362,7 @@
     <row r="182">
       <c r="A182" s="41" t="inlineStr">
         <is>
-          <t>Total equity – year 5</t>
+          <t>Total equity: year 5</t>
         </is>
       </c>
       <c r="F182" s="42">
@@ -5175,7 +5381,7 @@
     <row r="183">
       <c r="A183" s="41" t="inlineStr">
         <is>
-          <t>Diluted shares (000) – year 1</t>
+          <t>Diluted shares (000): year 1</t>
         </is>
       </c>
       <c r="F183" s="42">
@@ -5194,7 +5400,7 @@
     <row r="184">
       <c r="A184" s="41" t="inlineStr">
         <is>
-          <t>Diluted shares (000) – year 2</t>
+          <t>Diluted shares (000): year 2</t>
         </is>
       </c>
       <c r="F184" s="42">
@@ -5213,7 +5419,7 @@
     <row r="185">
       <c r="A185" s="41" t="inlineStr">
         <is>
-          <t>Diluted shares (000) – year 3</t>
+          <t>Diluted shares (000): year 3</t>
         </is>
       </c>
       <c r="F185" s="42">
@@ -5232,7 +5438,7 @@
     <row r="186">
       <c r="A186" s="41" t="inlineStr">
         <is>
-          <t>Diluted shares (000) – year 4</t>
+          <t>Diluted shares (000): year 4</t>
         </is>
       </c>
       <c r="F186" s="42">
@@ -5251,7 +5457,7 @@
     <row r="187">
       <c r="A187" s="41" t="inlineStr">
         <is>
-          <t>Diluted shares (000) – year 5</t>
+          <t>Diluted shares (000): year 5</t>
         </is>
       </c>
       <c r="F187" s="42">
@@ -5270,7 +5476,7 @@
     <row r="188">
       <c r="A188" s="41" t="inlineStr">
         <is>
-          <t>Diluted EPS ($) – year 1</t>
+          <t>Diluted EPS ($): year 1</t>
         </is>
       </c>
       <c r="F188" s="49">
@@ -5289,7 +5495,7 @@
     <row r="189">
       <c r="A189" s="41" t="inlineStr">
         <is>
-          <t>Diluted EPS ($) – year 2</t>
+          <t>Diluted EPS ($): year 2</t>
         </is>
       </c>
       <c r="F189" s="49">
@@ -5308,7 +5514,7 @@
     <row r="190">
       <c r="A190" s="41" t="inlineStr">
         <is>
-          <t>Diluted EPS ($) – year 3</t>
+          <t>Diluted EPS ($): year 3</t>
         </is>
       </c>
       <c r="F190" s="49">
@@ -5327,7 +5533,7 @@
     <row r="191">
       <c r="A191" s="41" t="inlineStr">
         <is>
-          <t>Diluted EPS ($) – year 4</t>
+          <t>Diluted EPS ($): year 4</t>
         </is>
       </c>
       <c r="F191" s="49">
@@ -5346,7 +5552,7 @@
     <row r="192">
       <c r="A192" s="41" t="inlineStr">
         <is>
-          <t>Diluted EPS ($) – year 5</t>
+          <t>Diluted EPS ($): year 5</t>
         </is>
       </c>
       <c r="F192" s="49">
@@ -5419,6 +5625,9 @@
         <v>11102600</v>
       </c>
     </row>
+    <row r="199"/>
+    <row r="200"/>
+    <row r="201"/>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add How it moves notes to Revenue Drivers tab
Add 38 short driver notes in column I (same colon-style as Scenarios),
covering store fleet, productivity, e-comm, geo/mix, and reconciliation.
Includes add_revenue_driver_notes.py for reproducibility.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/model18_wsp_formulas.xlsx
+++ b/LULU/model18_wsp_formulas.xlsx
@@ -458,7 +458,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="169">
+  <cellXfs count="170">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -914,6 +914,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="58" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -6575,7 +6578,7 @@
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="36" customWidth="1" min="9" max="9"/>
     <col width="28" customWidth="1" min="10" max="11"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="36" customWidth="1" min="12" max="12"/>
@@ -6684,7 +6687,11 @@
           <t>Units</t>
         </is>
       </c>
-      <c r="I5" s="56" t="n"/>
+      <c r="I5" s="169" t="inlineStr">
+        <is>
+          <t>How it moves</t>
+        </is>
+      </c>
       <c r="J5" s="127" t="inlineStr">
         <is>
           <t>Source</t>
@@ -6726,7 +6733,11 @@
           <t>stores</t>
         </is>
       </c>
-      <c r="I6" s="17" t="n"/>
+      <c r="I6" s="135" t="inlineStr">
+        <is>
+          <t>Prior-year ending count carried into this year.</t>
+        </is>
+      </c>
       <c r="J6" s="18" t="inlineStr">
         <is>
           <t>Revenue Drivers: beginning-stores formula</t>
@@ -6759,7 +6770,11 @@
           <t>stores</t>
         </is>
       </c>
-      <c r="I7" s="17" t="n"/>
+      <c r="I7" s="135" t="inlineStr">
+        <is>
+          <t>New stores added in region each forecast year.</t>
+        </is>
+      </c>
       <c r="J7" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: store count &amp; expansion</t>
@@ -6797,7 +6812,11 @@
           <t>stores</t>
         </is>
       </c>
-      <c r="I8" s="17" t="n"/>
+      <c r="I8" s="135" t="inlineStr">
+        <is>
+          <t>Stores closed yearly as leases roll off.</t>
+        </is>
+      </c>
       <c r="J8" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: lease renewal / fleet</t>
@@ -6843,7 +6862,11 @@
           <t>stores</t>
         </is>
       </c>
-      <c r="I9" s="17" t="n"/>
+      <c r="I9" s="135" t="inlineStr">
+        <is>
+          <t>Beginning plus openings minus closures each year.</t>
+        </is>
+      </c>
       <c r="J9" s="18" t="inlineStr">
         <is>
           <t>Revenue Drivers: ending-stores formula</t>
@@ -6884,7 +6907,11 @@
           <t>stores</t>
         </is>
       </c>
-      <c r="I10" s="17" t="n"/>
+      <c r="I10" s="135" t="inlineStr">
+        <is>
+          <t>Prior-year ending count carried into this year.</t>
+        </is>
+      </c>
       <c r="J10" s="18" t="inlineStr">
         <is>
           <t>Revenue Drivers: beginning-stores formula</t>
@@ -6917,7 +6944,11 @@
           <t>stores</t>
         </is>
       </c>
-      <c r="I11" s="17" t="n"/>
+      <c r="I11" s="135" t="inlineStr">
+        <is>
+          <t>New stores added in region each forecast year.</t>
+        </is>
+      </c>
       <c r="J11" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: store count &amp; expansion</t>
@@ -6955,7 +6986,11 @@
           <t>stores</t>
         </is>
       </c>
-      <c r="I12" s="17" t="n"/>
+      <c r="I12" s="135" t="inlineStr">
+        <is>
+          <t>Stores closed yearly as leases roll off.</t>
+        </is>
+      </c>
       <c r="J12" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: lease renewal / fleet</t>
@@ -7001,7 +7036,11 @@
           <t>stores</t>
         </is>
       </c>
-      <c r="I13" s="17" t="n"/>
+      <c r="I13" s="135" t="inlineStr">
+        <is>
+          <t>Beginning plus openings minus closures each year.</t>
+        </is>
+      </c>
       <c r="J13" s="18" t="inlineStr">
         <is>
           <t>Revenue Drivers: ending-stores formula</t>
@@ -7042,7 +7081,11 @@
           <t>stores</t>
         </is>
       </c>
-      <c r="I14" s="17" t="n"/>
+      <c r="I14" s="135" t="inlineStr">
+        <is>
+          <t>Prior-year ending count carried into this year.</t>
+        </is>
+      </c>
       <c r="J14" s="18" t="inlineStr">
         <is>
           <t>Revenue Drivers: beginning-stores formula</t>
@@ -7075,7 +7118,11 @@
           <t>stores</t>
         </is>
       </c>
-      <c r="I15" s="17" t="n"/>
+      <c r="I15" s="135" t="inlineStr">
+        <is>
+          <t>New stores added in region each forecast year.</t>
+        </is>
+      </c>
       <c r="J15" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: store count &amp; expansion</t>
@@ -7113,7 +7160,11 @@
           <t>stores</t>
         </is>
       </c>
-      <c r="I16" s="17" t="n"/>
+      <c r="I16" s="135" t="inlineStr">
+        <is>
+          <t>Stores closed yearly as leases roll off.</t>
+        </is>
+      </c>
       <c r="J16" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: lease renewal / fleet</t>
@@ -7159,7 +7210,11 @@
           <t>stores</t>
         </is>
       </c>
-      <c r="I17" s="17" t="n"/>
+      <c r="I17" s="135" t="inlineStr">
+        <is>
+          <t>Beginning plus openings minus closures each year.</t>
+        </is>
+      </c>
       <c r="J17" s="18" t="inlineStr">
         <is>
           <t>Revenue Drivers: ending-stores formula</t>
@@ -7195,7 +7250,11 @@
         <f>G9+G13+G17</f>
         <v/>
       </c>
-      <c r="I18" s="17" t="n"/>
+      <c r="I18" s="135" t="inlineStr">
+        <is>
+          <t>Sum of Americas, China, and Rest of World.</t>
+        </is>
+      </c>
       <c r="J18" s="18" t="inlineStr">
         <is>
           <t>Revenue Drivers: total-stores formula</t>
@@ -7231,7 +7290,11 @@
           <t>sq ft</t>
         </is>
       </c>
-      <c r="I19" s="17" t="n"/>
+      <c r="I19" s="135" t="inlineStr">
+        <is>
+          <t>Average box size grows modestly through FY30.</t>
+        </is>
+      </c>
       <c r="J19" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: sales per square foot</t>
@@ -7278,7 +7341,11 @@
           <t>sq ft</t>
         </is>
       </c>
-      <c r="I20" s="17" t="n"/>
+      <c r="I20" s="135" t="inlineStr">
+        <is>
+          <t>Ending stores times average square feet per store.</t>
+        </is>
+      </c>
       <c r="J20" s="128" t="inlineStr">
         <is>
           <t>Revenue Drivers: total-sqft formula</t>
@@ -7370,7 +7437,11 @@
           <t>$/sq ft</t>
         </is>
       </c>
-      <c r="I24" s="17" t="n"/>
+      <c r="I24" s="135" t="inlineStr">
+        <is>
+          <t>Sales per foot recovers slowly after FY26 trough.</t>
+        </is>
+      </c>
       <c r="J24" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: comparable sales &amp; SPSF</t>
@@ -7411,7 +7482,11 @@
           <t>%</t>
         </is>
       </c>
-      <c r="I25" s="17" t="n"/>
+      <c r="I25" s="135" t="inlineStr">
+        <is>
+          <t>Declines then flatlines as Americas traffic stabilizes.</t>
+        </is>
+      </c>
       <c r="J25" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: Americas comparable sales</t>
@@ -7452,7 +7527,11 @@
           <t>%</t>
         </is>
       </c>
-      <c r="I26" s="17" t="n"/>
+      <c r="I26" s="135" t="inlineStr">
+        <is>
+          <t>Strong growth moderates as China store base scales.</t>
+        </is>
+      </c>
       <c r="J26" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: China Mainland comparable sales</t>
@@ -7493,7 +7572,11 @@
           <t>%</t>
         </is>
       </c>
-      <c r="I27" s="17" t="n"/>
+      <c r="I27" s="135" t="inlineStr">
+        <is>
+          <t>Mid-single-digit comps fading to low-single digits.</t>
+        </is>
+      </c>
       <c r="J27" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: Rest of World comparable sales</t>
@@ -7539,7 +7622,11 @@
           <t>$000</t>
         </is>
       </c>
-      <c r="I28" s="17" t="n"/>
+      <c r="I28" s="135" t="inlineStr">
+        <is>
+          <t>Last year's store revenue rolled forward annually.</t>
+        </is>
+      </c>
       <c r="J28" s="18" t="inlineStr">
         <is>
           <t>Revenue Drivers: prior store-rev formula</t>
@@ -7575,7 +7662,11 @@
         <f>F28*0.71*(1+G25)+F28*0.16*(1+G26)+F28*0.13*(1+G27)</f>
         <v/>
       </c>
-      <c r="I29" s="17" t="n"/>
+      <c r="I29" s="135" t="inlineStr">
+        <is>
+          <t>Prior revenue grown by weighted geographic comp rates.</t>
+        </is>
+      </c>
       <c r="J29" s="18" t="inlineStr">
         <is>
           <t>Revenue Drivers: comp-store formula</t>
@@ -7611,7 +7702,11 @@
         <f>(G7-G8+G11-G12+G15-G16)*G19*G24/1000*0.55</f>
         <v/>
       </c>
-      <c r="I30" s="17" t="n"/>
+      <c r="I30" s="135" t="inlineStr">
+        <is>
+          <t>Net new doors times sq ft, productivity, ramp.</t>
+        </is>
+      </c>
       <c r="J30" s="128" t="inlineStr">
         <is>
           <t>Revenue Drivers: net-new-store formula</t>
@@ -7647,7 +7742,11 @@
         <f>G29+G30</f>
         <v/>
       </c>
-      <c r="I31" s="17" t="n"/>
+      <c r="I31" s="135" t="inlineStr">
+        <is>
+          <t>Comparable store sales plus new store contribution.</t>
+        </is>
+      </c>
       <c r="J31" s="18" t="inlineStr">
         <is>
           <t>Revenue Drivers: store-channel formula</t>
@@ -7840,7 +7939,11 @@
           <t>M</t>
         </is>
       </c>
-      <c r="I38" s="17" t="n"/>
+      <c r="I38" s="135" t="inlineStr">
+        <is>
+          <t>Digital traffic grows modestly across forecast years.</t>
+        </is>
+      </c>
       <c r="J38" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: e-commerce revenue</t>
@@ -7876,7 +7979,11 @@
       <c r="G39" s="64" t="n">
         <v>0.036</v>
       </c>
-      <c r="I39" s="17" t="n"/>
+      <c r="I39" s="135" t="inlineStr">
+        <is>
+          <t>Conversion rate recovers gradually from FY26 pressure.</t>
+        </is>
+      </c>
       <c r="J39" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: digital / traffic commentary</t>
@@ -7912,7 +8019,11 @@
       <c r="G40" s="67" t="n">
         <v>315</v>
       </c>
-      <c r="I40" s="17" t="n"/>
+      <c r="I40" s="135" t="inlineStr">
+        <is>
+          <t>Order size steps up slowly with promo normalization.</t>
+        </is>
+      </c>
       <c r="J40" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: e-commerce revenue</t>
@@ -7953,7 +8064,11 @@
         <f>G38*$B$3*G39*G40/$C$3</f>
         <v/>
       </c>
-      <c r="I41" s="17" t="n"/>
+      <c r="I41" s="135" t="inlineStr">
+        <is>
+          <t>Sessions times conversion times average order value.</t>
+        </is>
+      </c>
       <c r="J41" s="18" t="inlineStr">
         <is>
           <t>Revenue Drivers: e-comm formula</t>
@@ -8050,7 +8165,11 @@
           <t>$000</t>
         </is>
       </c>
-      <c r="I45" s="17" t="n"/>
+      <c r="I45" s="135" t="inlineStr">
+        <is>
+          <t>Wholesale, license, outlets: low-single-digit growth.</t>
+        </is>
+      </c>
       <c r="J45" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: channel revenue table</t>
@@ -8096,7 +8215,11 @@
           <t>$000</t>
         </is>
       </c>
-      <c r="I46" s="17" t="n"/>
+      <c r="I46" s="135" t="inlineStr">
+        <is>
+          <t>Americas revenue scales with consolidated growth rate.</t>
+        </is>
+      </c>
       <c r="J46" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: segmented net revenue</t>
@@ -8142,7 +8265,11 @@
           <t>$000</t>
         </is>
       </c>
-      <c r="I47" s="17" t="n"/>
+      <c r="I47" s="135" t="inlineStr">
+        <is>
+          <t>China revenue grows faster than consolidated average.</t>
+        </is>
+      </c>
       <c r="J47" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: segmented net revenue</t>
@@ -8188,7 +8315,11 @@
           <t>$000</t>
         </is>
       </c>
-      <c r="I48" s="17" t="n"/>
+      <c r="I48" s="135" t="inlineStr">
+        <is>
+          <t>Rest of World scales with total revenue growth.</t>
+        </is>
+      </c>
       <c r="J48" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: segmented net revenue</t>
@@ -8224,7 +8355,11 @@
       <c r="G49" s="64" t="n">
         <v>0.6</v>
       </c>
-      <c r="I49" s="17" t="n"/>
+      <c r="I49" s="135" t="inlineStr">
+        <is>
+          <t>Women's share fades slightly as men's mix rises.</t>
+        </is>
+      </c>
       <c r="J49" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: product category mix</t>
@@ -8260,7 +8395,11 @@
       <c r="G50" s="64" t="n">
         <v>0.27</v>
       </c>
-      <c r="I50" s="17" t="n"/>
+      <c r="I50" s="135" t="inlineStr">
+        <is>
+          <t>Men's mix rises gradually through the forecast.</t>
+        </is>
+      </c>
       <c r="J50" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: product category mix</t>
@@ -8296,7 +8435,11 @@
       <c r="G51" s="64" t="n">
         <v>0.13</v>
       </c>
-      <c r="I51" s="17" t="n"/>
+      <c r="I51" s="135" t="inlineStr">
+        <is>
+          <t>Accessories share held steady near thirteen percent.</t>
+        </is>
+      </c>
       <c r="J51" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: product category mix</t>
@@ -8393,7 +8536,11 @@
         <f>G31+G41+G45</f>
         <v/>
       </c>
-      <c r="I55" s="17" t="n"/>
+      <c r="I55" s="135" t="inlineStr">
+        <is>
+          <t>Store channel plus e-comm plus other channels.</t>
+        </is>
+      </c>
       <c r="J55" s="18" t="inlineStr">
         <is>
           <t>Revenue Drivers: total-rev formula</t>
@@ -8429,7 +8576,11 @@
         <f>Scenarios!$C$29</f>
         <v/>
       </c>
-      <c r="I56" s="17" t="n"/>
+      <c r="I56" s="135" t="inlineStr">
+        <is>
+          <t>Pulls Scenarios base revenue path used by DCF.</t>
+        </is>
+      </c>
       <c r="J56" s="18" t="inlineStr">
         <is>
           <t>Scenarios tab: base revenue</t>
@@ -8471,7 +8622,11 @@
         <f>G55-G56</f>
         <v/>
       </c>
-      <c r="I57" s="17" t="n"/>
+      <c r="I57" s="135" t="inlineStr">
+        <is>
+          <t>Driver-built revenue minus Scenarios base-case revenue.</t>
+        </is>
+      </c>
       <c r="J57" s="128" t="inlineStr">
         <is>
           <t>Revenue Drivers: variance formula</t>
@@ -8508,7 +8663,11 @@
         <f>IF(G56=0,"",G57/G56)</f>
         <v/>
       </c>
-      <c r="I58" s="17" t="n"/>
+      <c r="I58" s="135" t="inlineStr">
+        <is>
+          <t>Variance as percent of Scenarios consolidated revenue.</t>
+        </is>
+      </c>
       <c r="J58" s="128" t="inlineStr">
         <is>
           <t>Revenue Drivers: variance % formula</t>

</xml_diff>

<commit_message>
Fix DCF repurchase EPS to match Scenarios; sync deck EPS callouts
- Link DCF repurchase schedule (rows 75/77/78, cols F-J) to Scenarios
  pitch bridge so Share Repurchase & EPS Accretion Schedule matches slides
- Harden update_pitch_numbers_only.py: regex EPS patches on slides 12-14,
  fix bear/bull double-replace typo (202.17.17), stale 14.57/14.87 swaps
- recalc_model18 reads EPS from DCF row 78 when available

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/model18_wsp_formulas.xlsx
+++ b/LULU/model18_wsp_formulas.xlsx
@@ -10398,23 +10398,23 @@
         <v>111380</v>
       </c>
       <c r="F75" s="25">
-        <f>F74-F73</f>
+        <f>Scenarios!$C$183</f>
         <v/>
       </c>
       <c r="G75" s="25">
-        <f>G74-G73</f>
+        <f>Scenarios!$C$184</f>
         <v/>
       </c>
       <c r="H75" s="25">
-        <f>H74-H73</f>
+        <f>Scenarios!$C$185</f>
         <v/>
       </c>
       <c r="I75" s="25">
-        <f>I74-I73</f>
+        <f>Scenarios!$C$186</f>
         <v/>
       </c>
       <c r="J75" s="25">
-        <f>J74-J73</f>
+        <f>Scenarios!$C$187</f>
         <v/>
       </c>
     </row>
@@ -10428,23 +10428,23 @@
         <v>1579183</v>
       </c>
       <c r="F77" s="75">
-        <f>F14</f>
+        <f>Scenarios!$C$143</f>
         <v/>
       </c>
       <c r="G77" s="75">
-        <f>G14</f>
+        <f>Scenarios!$C$144</f>
         <v/>
       </c>
       <c r="H77" s="75">
-        <f>H14</f>
+        <f>Scenarios!$C$145</f>
         <v/>
       </c>
       <c r="I77" s="75">
-        <f>I14</f>
+        <f>Scenarios!$C$146</f>
         <v/>
       </c>
       <c r="J77" s="75">
-        <f>J14</f>
+        <f>Scenarios!$C$147</f>
         <v/>
       </c>
     </row>
@@ -10459,23 +10459,23 @@
         <v/>
       </c>
       <c r="F78" s="101">
-        <f>F77/F75</f>
+        <f>Scenarios!$C$188</f>
         <v/>
       </c>
       <c r="G78" s="101">
-        <f>G77/G75</f>
+        <f>Scenarios!$C$189</f>
         <v/>
       </c>
       <c r="H78" s="101">
-        <f>H77/H75</f>
+        <f>Scenarios!$C$190</f>
         <v/>
       </c>
       <c r="I78" s="101">
-        <f>I77/I75</f>
+        <f>Scenarios!$C$191</f>
         <v/>
       </c>
       <c r="J78" s="101">
-        <f>J77/J75</f>
+        <f>Scenarios!$C$192</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix DCF WACC×g sensitivity grid — wrong TV discount exponent
Cols F-H referenced empty E36 (^0 = no TV discount); cols I-J kept
stale hardcoded ^5 formulas. All five g columns now use ^$J$36 (=5).

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/model18_wsp_formulas.xlsx
+++ b/LULU/model18_wsp_formulas.xlsx
@@ -10713,23 +10713,23 @@
       </c>
       <c r="D99" s="19" t="n"/>
       <c r="F99" s="110">
-        <f>(NPV($A99,$F$35:$J$35)+($J$35*(1+F$98)/($A99-F$98))/(1+$A99)^$E$36+$E$50+$E$51)/$E$55</f>
+        <f>(NPV($A99,$F$35:$J$35)+($J$35*(1+F$98)/($A99-F$98))/(1+$A99)^$J$36+$E$50+$E$51)/$E$55</f>
         <v/>
       </c>
       <c r="G99" s="110">
-        <f>(NPV($A99,$F$35:$J$35)+($J$35*(1+G$98)/($A99-G$98))/(1+$A99)^$E$36+$E$50+$E$51)/$E$55</f>
+        <f>(NPV($A99,$F$35:$J$35)+($J$35*(1+G$98)/($A99-G$98))/(1+$A99)^$J$36+$E$50+$E$51)/$E$55</f>
         <v/>
       </c>
       <c r="H99" s="110">
-        <f>(NPV($A99,$F$35:$J$35)+($J$35*(1+H$98)/($A99-H$98))/(1+$A99)^$E$36+$E$50+$E$51)/$E$55</f>
+        <f>(NPV($A99,$F$35:$J$35)+($J$35*(1+H$98)/($A99-H$98))/(1+$A99)^$J$36+$E$50+$E$51)/$E$55</f>
         <v/>
       </c>
       <c r="I99" s="110">
-        <f>(NPV(0.095,F35:J35)+(J35*(1+0.025)/(0.095-0.025))/(1+0.095)^5+E50+E51)/E55</f>
+        <f>(NPV($A99,$F$35:$J$35)+($J$35*(1+I$98)/($A99-I$98))/(1+$A99)^$J$36+$E$50+$E$51)/$E$55</f>
         <v/>
       </c>
       <c r="J99" s="110">
-        <f>(NPV(0.095,F35:J35)+(J35*(1+0.03)/(0.095-0.03))/(1+0.095)^5+E50+E51)/E55</f>
+        <f>(NPV($A99,$F$35:$J$35)+($J$35*(1+J$98)/($A99-J$98))/(1+$A99)^$J$36+$E$50+$E$51)/$E$55</f>
         <v/>
       </c>
     </row>
@@ -10739,23 +10739,23 @@
       </c>
       <c r="D100" s="19" t="n"/>
       <c r="F100" s="110">
-        <f>(NPV($A100,$F$35:$J$35)+($J$35*(1+F$98)/($A100-F$98))/(1+$A100)^$E$36+$E$50+$E$51)/$E$55</f>
+        <f>(NPV($A100,$F$35:$J$35)+($J$35*(1+F$98)/($A100-F$98))/(1+$A100)^$J$36+$E$50+$E$51)/$E$55</f>
         <v/>
       </c>
       <c r="G100" s="110">
-        <f>(NPV($A100,$F$35:$J$35)+($J$35*(1+G$98)/($A100-G$98))/(1+$A100)^$E$36+$E$50+$E$51)/$E$55</f>
+        <f>(NPV($A100,$F$35:$J$35)+($J$35*(1+G$98)/($A100-G$98))/(1+$A100)^$J$36+$E$50+$E$51)/$E$55</f>
         <v/>
       </c>
       <c r="H100" s="110">
-        <f>(NPV($A100,$F$35:$J$35)+($J$35*(1+H$98)/($A100-H$98))/(1+$A100)^$E$36+$E$50+$E$51)/$E$55</f>
+        <f>(NPV($A100,$F$35:$J$35)+($J$35*(1+H$98)/($A100-H$98))/(1+$A100)^$J$36+$E$50+$E$51)/$E$55</f>
         <v/>
       </c>
       <c r="I100" s="110">
-        <f>(NPV(0.1,F35:J35)+(J35*(1+0.025)/(0.1-0.025))/(1+0.1)^5+E50+E51)/E55</f>
+        <f>(NPV($A100,$F$35:$J$35)+($J$35*(1+I$98)/($A100-I$98))/(1+$A100)^$J$36+$E$50+$E$51)/$E$55</f>
         <v/>
       </c>
       <c r="J100" s="110">
-        <f>(NPV(0.1,F35:J35)+(J35*(1+0.03)/(0.1-0.03))/(1+0.1)^5+E50+E51)/E55</f>
+        <f>(NPV($A100,$F$35:$J$35)+($J$35*(1+J$98)/($A100-J$98))/(1+$A100)^$J$36+$E$50+$E$51)/$E$55</f>
         <v/>
       </c>
     </row>
@@ -10765,23 +10765,23 @@
       </c>
       <c r="D101" s="19" t="n"/>
       <c r="F101" s="110">
-        <f>(NPV($A101,$F$35:$J$35)+($J$35*(1+F$98)/($A101-F$98))/(1+$A101)^$E$36+$E$50+$E$51)/$E$55</f>
+        <f>(NPV($A101,$F$35:$J$35)+($J$35*(1+F$98)/($A101-F$98))/(1+$A101)^$J$36+$E$50+$E$51)/$E$55</f>
         <v/>
       </c>
       <c r="G101" s="110">
-        <f>(NPV($A101,$F$35:$J$35)+($J$35*(1+G$98)/($A101-G$98))/(1+$A101)^$E$36+$E$50+$E$51)/$E$55</f>
+        <f>(NPV($A101,$F$35:$J$35)+($J$35*(1+G$98)/($A101-G$98))/(1+$A101)^$J$36+$E$50+$E$51)/$E$55</f>
         <v/>
       </c>
       <c r="H101" s="111">
-        <f>(NPV($A101,$F$35:$J$35)+($J$35*(1+H$98)/($A101-H$98))/(1+$A101)^$E$36+$E$50+$E$51)/$E$55</f>
+        <f>(NPV($A101,$F$35:$J$35)+($J$35*(1+H$98)/($A101-H$98))/(1+$A101)^$J$36+$E$50+$E$51)/$E$55</f>
         <v/>
       </c>
       <c r="I101" s="110">
-        <f>(NPV(0.105,F35:J35)+(J35*(1+0.025)/(0.105-0.025))/(1+0.105)^5+E50+E51)/E55</f>
+        <f>(NPV($A101,$F$35:$J$35)+($J$35*(1+I$98)/($A101-I$98))/(1+$A101)^$J$36+$E$50+$E$51)/$E$55</f>
         <v/>
       </c>
       <c r="J101" s="110">
-        <f>(NPV(0.105,F35:J35)+(J35*(1+0.03)/(0.105-0.03))/(1+0.105)^5+E50+E51)/E55</f>
+        <f>(NPV($A101,$F$35:$J$35)+($J$35*(1+J$98)/($A101-J$98))/(1+$A101)^$J$36+$E$50+$E$51)/$E$55</f>
         <v/>
       </c>
     </row>
@@ -10791,23 +10791,23 @@
       </c>
       <c r="D102" s="19" t="n"/>
       <c r="F102" s="110">
-        <f>(NPV($A102,$F$35:$J$35)+($J$35*(1+F$98)/($A102-F$98))/(1+$A102)^$E$36+$E$50+$E$51)/$E$55</f>
+        <f>(NPV($A102,$F$35:$J$35)+($J$35*(1+F$98)/($A102-F$98))/(1+$A102)^$J$36+$E$50+$E$51)/$E$55</f>
         <v/>
       </c>
       <c r="G102" s="110">
-        <f>(NPV($A102,$F$35:$J$35)+($J$35*(1+G$98)/($A102-G$98))/(1+$A102)^$E$36+$E$50+$E$51)/$E$55</f>
+        <f>(NPV($A102,$F$35:$J$35)+($J$35*(1+G$98)/($A102-G$98))/(1+$A102)^$J$36+$E$50+$E$51)/$E$55</f>
         <v/>
       </c>
       <c r="H102" s="110">
-        <f>(NPV($A102,$F$35:$J$35)+($J$35*(1+H$98)/($A102-H$98))/(1+$A102)^$E$36+$E$50+$E$51)/$E$55</f>
+        <f>(NPV($A102,$F$35:$J$35)+($J$35*(1+H$98)/($A102-H$98))/(1+$A102)^$J$36+$E$50+$E$51)/$E$55</f>
         <v/>
       </c>
       <c r="I102" s="110">
-        <f>(NPV(0.11,F35:J35)+(J35*(1+0.025)/(0.11-0.025))/(1+0.11)^5+E50+E51)/E55</f>
+        <f>(NPV($A102,$F$35:$J$35)+($J$35*(1+I$98)/($A102-I$98))/(1+$A102)^$J$36+$E$50+$E$51)/$E$55</f>
         <v/>
       </c>
       <c r="J102" s="110">
-        <f>(NPV(0.11,F35:J35)+(J35*(1+0.03)/(0.11-0.03))/(1+0.11)^5+E50+E51)/E55</f>
+        <f>(NPV($A102,$F$35:$J$35)+($J$35*(1+J$98)/($A102-J$98))/(1+$A102)^$J$36+$E$50+$E$51)/$E$55</f>
         <v/>
       </c>
     </row>
@@ -10817,23 +10817,23 @@
       </c>
       <c r="D103" s="19" t="n"/>
       <c r="F103" s="110">
-        <f>(NPV($A103,$F$35:$J$35)+($J$35*(1+F$98)/($A103-F$98))/(1+$A103)^$E$36+$E$50+$E$51)/$E$55</f>
+        <f>(NPV($A103,$F$35:$J$35)+($J$35*(1+F$98)/($A103-F$98))/(1+$A103)^$J$36+$E$50+$E$51)/$E$55</f>
         <v/>
       </c>
       <c r="G103" s="110">
-        <f>(NPV($A103,$F$35:$J$35)+($J$35*(1+G$98)/($A103-G$98))/(1+$A103)^$E$36+$E$50+$E$51)/$E$55</f>
+        <f>(NPV($A103,$F$35:$J$35)+($J$35*(1+G$98)/($A103-G$98))/(1+$A103)^$J$36+$E$50+$E$51)/$E$55</f>
         <v/>
       </c>
       <c r="H103" s="110">
-        <f>(NPV($A103,$F$35:$J$35)+($J$35*(1+H$98)/($A103-H$98))/(1+$A103)^$E$36+$E$50+$E$51)/$E$55</f>
+        <f>(NPV($A103,$F$35:$J$35)+($J$35*(1+H$98)/($A103-H$98))/(1+$A103)^$J$36+$E$50+$E$51)/$E$55</f>
         <v/>
       </c>
       <c r="I103" s="110">
-        <f>(NPV(0.115,F35:J35)+(J35*(1+0.025)/(0.115-0.025))/(1+0.115)^5+E50+E51)/E55</f>
+        <f>(NPV($A103,$F$35:$J$35)+($J$35*(1+I$98)/($A103-I$98))/(1+$A103)^$J$36+$E$50+$E$51)/$E$55</f>
         <v/>
       </c>
       <c r="J103" s="110">
-        <f>(NPV(0.115,F35:J35)+(J35*(1+0.03)/(0.115-0.03))/(1+0.115)^5+E50+E51)/E55</f>
+        <f>(NPV($A103,$F$35:$J$35)+($J$35*(1+J$98)/($A103-J$98))/(1+$A103)^$J$36+$E$50+$E$51)/$E$55</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove duplicate FY25 anchor values in Scenarios column F (rows 194-203)
Column B is the canonical anchor (Scenarios!$B$194 etc.); column F copies were unreferenced leftovers.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/model18_wsp_formulas.xlsx
+++ b/LULU/model18_wsp_formulas.xlsx
@@ -6638,9 +6638,7 @@
       <c r="C194" s="174" t="n"/>
       <c r="D194" s="174" t="n"/>
       <c r="E194" s="174" t="n"/>
-      <c r="F194" s="174" t="n">
-        <v>8456743</v>
-      </c>
+      <c r="F194" s="174" t="n"/>
       <c r="G194" s="171" t="n"/>
       <c r="H194" s="171" t="n"/>
     </row>
@@ -6656,9 +6654,7 @@
       <c r="C195" s="174" t="n"/>
       <c r="D195" s="174" t="n"/>
       <c r="E195" s="174" t="n"/>
-      <c r="F195" s="174" t="n">
-        <v>3494903</v>
-      </c>
+      <c r="F195" s="174" t="n"/>
       <c r="G195" s="171" t="n"/>
       <c r="H195" s="171" t="n"/>
     </row>
@@ -6674,9 +6670,7 @@
       <c r="C196" s="174" t="n"/>
       <c r="D196" s="174" t="n"/>
       <c r="E196" s="174" t="n"/>
-      <c r="F196" s="174" t="n">
-        <v>4961840</v>
-      </c>
+      <c r="F196" s="174" t="n"/>
       <c r="G196" s="171" t="n"/>
       <c r="H196" s="171" t="n"/>
     </row>
@@ -6692,9 +6686,7 @@
       <c r="C197" s="174" t="n"/>
       <c r="D197" s="174" t="n"/>
       <c r="E197" s="174" t="n"/>
-      <c r="F197" s="174" t="n">
-        <v>119068</v>
-      </c>
+      <c r="F197" s="174" t="n"/>
       <c r="G197" s="171" t="n"/>
       <c r="H197" s="171" t="n"/>
     </row>
@@ -6710,9 +6702,7 @@
       <c r="C198" s="174" t="n"/>
       <c r="D198" s="174" t="n"/>
       <c r="E198" s="174" t="n"/>
-      <c r="F198" s="174" t="n">
-        <v>11102600</v>
-      </c>
+      <c r="F198" s="174" t="n"/>
       <c r="G198" s="171" t="n"/>
       <c r="H198" s="171" t="n"/>
     </row>
@@ -6758,9 +6748,7 @@
       <c r="C202" s="174" t="n"/>
       <c r="D202" s="174" t="n"/>
       <c r="E202" s="174" t="n"/>
-      <c r="F202" s="174" t="n">
-        <v>62203</v>
-      </c>
+      <c r="F202" s="174" t="n"/>
       <c r="G202" s="171" t="n"/>
       <c r="H202" s="171" t="n"/>
     </row>
@@ -6776,9 +6764,7 @@
       <c r="C203" s="174" t="n"/>
       <c r="D203" s="174" t="n"/>
       <c r="E203" s="174" t="n"/>
-      <c r="F203" s="174" t="n">
-        <v>1028</v>
-      </c>
+      <c r="F203" s="174" t="n"/>
       <c r="G203" s="171" t="n"/>
       <c r="H203" s="171" t="n"/>
     </row>

</xml_diff>